<commit_message>
Add File Edit EditProfile 11/11
</commit_message>
<xml_diff>
--- a/ExcelProject/Register Student.xlsx
+++ b/ExcelProject/Register Student.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1034" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1046" uniqueCount="285">
   <si>
     <t>Execute</t>
   </si>
@@ -827,7 +827,7 @@
     <t>Profile.docx</t>
   </si>
   <si>
-    <t>* ไฟล์ต้องเป็น .jpg, .jpeg, .png หรือ .gif เท่านั้น</t>
+    <t>ไฟล์ต้องเป็น .jpg, .jpeg, .png หรือ .gif เท่านั้น</t>
   </si>
   <si>
     <t>TC2:76</t>
@@ -857,7 +857,7 @@
     <t>Profile3.jpg</t>
   </si>
   <si>
-    <t>* ขนาดไฟล์ต้องไม่เกิน 5MB</t>
+    <t>ขนาดไฟล์ต้องไม่เกิน 5MB</t>
   </si>
   <si>
     <t>TC2:79</t>
@@ -866,7 +866,10 @@
     <t>MJU6504106454</t>
   </si>
   <si>
-    <t>* กรุณาเลือกไฟล์รูปภาพ</t>
+    <t>กรุณาเลือกไฟล์รูปภาพ</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -958,7 +961,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="27">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -997,6 +1000,24 @@
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
@@ -1325,20 +1346,20 @@
   <dimension ref="A1:N97"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="17" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="18" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="19" width="12.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="18" width="9.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="19" width="8.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="20" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="18" width="10.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="18" width="19.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="18" width="12.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="18" width="9.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="18" width="48.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="18" width="41.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="18" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="18" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="23" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="24" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="25" width="12.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="24" width="9.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="25" width="8.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="26" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="24" width="10.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="24" width="19.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="24" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="24" width="9.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="24" width="48.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="24" width="41.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="24" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="24" width="14.147857142857141" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="21.75">
@@ -2393,7 +2414,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="21.75">
       <c r="A25" s="4" t="s">
         <v>14</v>
       </c>
@@ -2437,7 +2458,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="21.75">
       <c r="A26" s="4" t="s">
         <v>14</v>
       </c>
@@ -2481,7 +2502,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="21.75">
       <c r="A27" s="4" t="s">
         <v>14</v>
       </c>
@@ -2525,7 +2546,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="21.75">
       <c r="A28" s="4" t="s">
         <v>14</v>
       </c>
@@ -2569,7 +2590,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="21.75">
       <c r="A29" s="4" t="s">
         <v>14</v>
       </c>
@@ -2613,7 +2634,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="21.75">
       <c r="A30" s="4" t="s">
         <v>14</v>
       </c>
@@ -2657,7 +2678,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="21.75">
       <c r="A31" s="4" t="s">
         <v>14</v>
       </c>
@@ -2701,7 +2722,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="21.75">
       <c r="A32" s="4" t="s">
         <v>14</v>
       </c>
@@ -2745,7 +2766,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="21.75">
       <c r="A33" s="4" t="s">
         <v>14</v>
       </c>
@@ -2789,7 +2810,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="21.75">
       <c r="A34" s="4" t="s">
         <v>14</v>
       </c>
@@ -4233,7 +4254,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="21.75">
       <c r="A67" s="4" t="s">
         <v>14</v>
       </c>
@@ -4277,7 +4298,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="21.75">
       <c r="A68" s="4" t="s">
         <v>14</v>
       </c>
@@ -4321,7 +4342,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="21.75">
       <c r="A69" s="4" t="s">
         <v>14</v>
       </c>
@@ -4365,7 +4386,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="21.75">
       <c r="A70" s="4" t="s">
         <v>14</v>
       </c>
@@ -4409,7 +4430,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="21.75">
       <c r="A71" s="4" t="s">
         <v>14</v>
       </c>
@@ -4453,7 +4474,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="21.75">
       <c r="A72" s="4" t="s">
         <v>14</v>
       </c>
@@ -4497,7 +4518,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="21.75">
       <c r="A73" s="4" t="s">
         <v>14</v>
       </c>
@@ -4541,7 +4562,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="21.75">
       <c r="A74" s="4" t="s">
         <v>14</v>
       </c>
@@ -4583,7 +4604,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="21.75">
       <c r="A75" s="4" t="s">
         <v>14</v>
       </c>
@@ -4627,7 +4648,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="21.75">
       <c r="A76" s="4" t="s">
         <v>14</v>
       </c>
@@ -4671,7 +4692,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="21.75">
       <c r="A77" s="4" t="s">
         <v>14</v>
       </c>
@@ -4803,7 +4824,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="22.5">
+    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="21.75">
       <c r="A80" s="4" t="s">
         <v>14</v>
       </c>
@@ -4845,277 +4866,301 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="19.5">
-      <c r="A81" s="14"/>
-      <c r="B81" s="15"/>
-      <c r="C81" s="15"/>
-      <c r="D81" s="15"/>
-      <c r="E81" s="15"/>
-      <c r="F81" s="16"/>
-      <c r="G81" s="15"/>
-      <c r="H81" s="15"/>
-      <c r="I81" s="15"/>
-      <c r="J81" s="15"/>
-      <c r="K81" s="15"/>
-      <c r="L81" s="15"/>
-      <c r="M81" s="15"/>
-      <c r="N81" s="15"/>
+    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="22.5">
+      <c r="A81" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="B81" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="C81" s="2"/>
+      <c r="D81" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="E81" s="16" t="s">
+        <v>284</v>
+      </c>
+      <c r="F81" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="G81" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="H81" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="I81" s="18" t="s">
+        <v>284</v>
+      </c>
+      <c r="J81" s="19" t="s">
+        <v>284</v>
+      </c>
+      <c r="K81" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="L81" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="M81" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="N81" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="19.5">
-      <c r="A82" s="14"/>
-      <c r="B82" s="15"/>
-      <c r="C82" s="15"/>
-      <c r="D82" s="15"/>
-      <c r="E82" s="15"/>
-      <c r="F82" s="16"/>
-      <c r="G82" s="15"/>
-      <c r="H82" s="15"/>
-      <c r="I82" s="15"/>
-      <c r="J82" s="15"/>
-      <c r="K82" s="15"/>
-      <c r="L82" s="15"/>
-      <c r="M82" s="15"/>
-      <c r="N82" s="15"/>
+      <c r="A82" s="20"/>
+      <c r="B82" s="21"/>
+      <c r="C82" s="21"/>
+      <c r="D82" s="21"/>
+      <c r="E82" s="21"/>
+      <c r="F82" s="22"/>
+      <c r="G82" s="21"/>
+      <c r="H82" s="21"/>
+      <c r="I82" s="21"/>
+      <c r="J82" s="21"/>
+      <c r="K82" s="21"/>
+      <c r="L82" s="21"/>
+      <c r="M82" s="21"/>
+      <c r="N82" s="21"/>
     </row>
     <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="19.5">
-      <c r="A83" s="14"/>
-      <c r="B83" s="15"/>
-      <c r="C83" s="15"/>
-      <c r="D83" s="15"/>
-      <c r="E83" s="15"/>
-      <c r="F83" s="16"/>
-      <c r="G83" s="15"/>
-      <c r="H83" s="15"/>
-      <c r="I83" s="15"/>
-      <c r="J83" s="15"/>
-      <c r="K83" s="15"/>
-      <c r="L83" s="15"/>
-      <c r="M83" s="15"/>
-      <c r="N83" s="15"/>
+      <c r="A83" s="20"/>
+      <c r="B83" s="21"/>
+      <c r="C83" s="21"/>
+      <c r="D83" s="21"/>
+      <c r="E83" s="21"/>
+      <c r="F83" s="22"/>
+      <c r="G83" s="21"/>
+      <c r="H83" s="21"/>
+      <c r="I83" s="21"/>
+      <c r="J83" s="21"/>
+      <c r="K83" s="21"/>
+      <c r="L83" s="21"/>
+      <c r="M83" s="21"/>
+      <c r="N83" s="21"/>
     </row>
     <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="19.5">
-      <c r="A84" s="14"/>
-      <c r="B84" s="15"/>
-      <c r="C84" s="15"/>
-      <c r="D84" s="15"/>
-      <c r="E84" s="15"/>
-      <c r="F84" s="16"/>
-      <c r="G84" s="15"/>
-      <c r="H84" s="15"/>
-      <c r="I84" s="15"/>
-      <c r="J84" s="15"/>
-      <c r="K84" s="15"/>
-      <c r="L84" s="15"/>
-      <c r="M84" s="15"/>
-      <c r="N84" s="15"/>
+      <c r="A84" s="20"/>
+      <c r="B84" s="21"/>
+      <c r="C84" s="21"/>
+      <c r="D84" s="21"/>
+      <c r="E84" s="21"/>
+      <c r="F84" s="22"/>
+      <c r="G84" s="21"/>
+      <c r="H84" s="21"/>
+      <c r="I84" s="21"/>
+      <c r="J84" s="21"/>
+      <c r="K84" s="21"/>
+      <c r="L84" s="21"/>
+      <c r="M84" s="21"/>
+      <c r="N84" s="21"/>
     </row>
     <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="19.5">
-      <c r="A85" s="14"/>
-      <c r="B85" s="15"/>
-      <c r="C85" s="15"/>
-      <c r="D85" s="15"/>
-      <c r="E85" s="15"/>
-      <c r="F85" s="16"/>
-      <c r="G85" s="15"/>
-      <c r="H85" s="15"/>
-      <c r="I85" s="15"/>
-      <c r="J85" s="15"/>
-      <c r="K85" s="15"/>
-      <c r="L85" s="15"/>
-      <c r="M85" s="15"/>
-      <c r="N85" s="15"/>
+      <c r="A85" s="20"/>
+      <c r="B85" s="21"/>
+      <c r="C85" s="21"/>
+      <c r="D85" s="21"/>
+      <c r="E85" s="21"/>
+      <c r="F85" s="22"/>
+      <c r="G85" s="21"/>
+      <c r="H85" s="21"/>
+      <c r="I85" s="21"/>
+      <c r="J85" s="21"/>
+      <c r="K85" s="21"/>
+      <c r="L85" s="21"/>
+      <c r="M85" s="21"/>
+      <c r="N85" s="21"/>
     </row>
     <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="19.5">
-      <c r="A86" s="14"/>
-      <c r="B86" s="15"/>
-      <c r="C86" s="15"/>
-      <c r="D86" s="15"/>
-      <c r="E86" s="15"/>
-      <c r="F86" s="16"/>
-      <c r="G86" s="15"/>
-      <c r="H86" s="15"/>
-      <c r="I86" s="15"/>
-      <c r="J86" s="15"/>
-      <c r="K86" s="15"/>
-      <c r="L86" s="15"/>
-      <c r="M86" s="15"/>
-      <c r="N86" s="15"/>
+      <c r="A86" s="20"/>
+      <c r="B86" s="21"/>
+      <c r="C86" s="21"/>
+      <c r="D86" s="21"/>
+      <c r="E86" s="21"/>
+      <c r="F86" s="22"/>
+      <c r="G86" s="21"/>
+      <c r="H86" s="21"/>
+      <c r="I86" s="21"/>
+      <c r="J86" s="21"/>
+      <c r="K86" s="21"/>
+      <c r="L86" s="21"/>
+      <c r="M86" s="21"/>
+      <c r="N86" s="21"/>
     </row>
     <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="19.5">
-      <c r="A87" s="14"/>
-      <c r="B87" s="15"/>
-      <c r="C87" s="15"/>
-      <c r="D87" s="15"/>
-      <c r="E87" s="15"/>
-      <c r="F87" s="16"/>
-      <c r="G87" s="15"/>
-      <c r="H87" s="15"/>
-      <c r="I87" s="15"/>
-      <c r="J87" s="15"/>
-      <c r="K87" s="15"/>
-      <c r="L87" s="15"/>
-      <c r="M87" s="15"/>
-      <c r="N87" s="15"/>
+      <c r="A87" s="20"/>
+      <c r="B87" s="21"/>
+      <c r="C87" s="21"/>
+      <c r="D87" s="21"/>
+      <c r="E87" s="21"/>
+      <c r="F87" s="22"/>
+      <c r="G87" s="21"/>
+      <c r="H87" s="21"/>
+      <c r="I87" s="21"/>
+      <c r="J87" s="21"/>
+      <c r="K87" s="21"/>
+      <c r="L87" s="21"/>
+      <c r="M87" s="21"/>
+      <c r="N87" s="21"/>
     </row>
     <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="19.5">
-      <c r="A88" s="14"/>
-      <c r="B88" s="15"/>
-      <c r="C88" s="15"/>
-      <c r="D88" s="15"/>
-      <c r="E88" s="15"/>
-      <c r="F88" s="16"/>
-      <c r="G88" s="15"/>
-      <c r="H88" s="15"/>
-      <c r="I88" s="15"/>
-      <c r="J88" s="15"/>
-      <c r="K88" s="15"/>
-      <c r="L88" s="15"/>
-      <c r="M88" s="15"/>
-      <c r="N88" s="15"/>
+      <c r="A88" s="20"/>
+      <c r="B88" s="21"/>
+      <c r="C88" s="21"/>
+      <c r="D88" s="21"/>
+      <c r="E88" s="21"/>
+      <c r="F88" s="22"/>
+      <c r="G88" s="21"/>
+      <c r="H88" s="21"/>
+      <c r="I88" s="21"/>
+      <c r="J88" s="21"/>
+      <c r="K88" s="21"/>
+      <c r="L88" s="21"/>
+      <c r="M88" s="21"/>
+      <c r="N88" s="21"/>
     </row>
     <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="19.5">
-      <c r="A89" s="14"/>
-      <c r="B89" s="15"/>
-      <c r="C89" s="15"/>
-      <c r="D89" s="15"/>
-      <c r="E89" s="15"/>
-      <c r="F89" s="16"/>
-      <c r="G89" s="15"/>
-      <c r="H89" s="15"/>
-      <c r="I89" s="15"/>
-      <c r="J89" s="15"/>
-      <c r="K89" s="15"/>
-      <c r="L89" s="15"/>
-      <c r="M89" s="15"/>
-      <c r="N89" s="15"/>
+      <c r="A89" s="20"/>
+      <c r="B89" s="21"/>
+      <c r="C89" s="21"/>
+      <c r="D89" s="21"/>
+      <c r="E89" s="21"/>
+      <c r="F89" s="22"/>
+      <c r="G89" s="21"/>
+      <c r="H89" s="21"/>
+      <c r="I89" s="21"/>
+      <c r="J89" s="21"/>
+      <c r="K89" s="21"/>
+      <c r="L89" s="21"/>
+      <c r="M89" s="21"/>
+      <c r="N89" s="21"/>
     </row>
     <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="19.5">
-      <c r="A90" s="14"/>
-      <c r="B90" s="15"/>
-      <c r="C90" s="15"/>
-      <c r="D90" s="15"/>
-      <c r="E90" s="15"/>
-      <c r="F90" s="16"/>
-      <c r="G90" s="15"/>
-      <c r="H90" s="15"/>
-      <c r="I90" s="15"/>
-      <c r="J90" s="15"/>
-      <c r="K90" s="15"/>
-      <c r="L90" s="15"/>
-      <c r="M90" s="15"/>
-      <c r="N90" s="15"/>
+      <c r="A90" s="20"/>
+      <c r="B90" s="21"/>
+      <c r="C90" s="21"/>
+      <c r="D90" s="21"/>
+      <c r="E90" s="21"/>
+      <c r="F90" s="22"/>
+      <c r="G90" s="21"/>
+      <c r="H90" s="21"/>
+      <c r="I90" s="21"/>
+      <c r="J90" s="21"/>
+      <c r="K90" s="21"/>
+      <c r="L90" s="21"/>
+      <c r="M90" s="21"/>
+      <c r="N90" s="21"/>
     </row>
     <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="19.5">
-      <c r="A91" s="14"/>
-      <c r="B91" s="15"/>
-      <c r="C91" s="15"/>
-      <c r="D91" s="15"/>
-      <c r="E91" s="15"/>
-      <c r="F91" s="16"/>
-      <c r="G91" s="15"/>
-      <c r="H91" s="15"/>
-      <c r="I91" s="15"/>
-      <c r="J91" s="15"/>
-      <c r="K91" s="15"/>
-      <c r="L91" s="15"/>
-      <c r="M91" s="15"/>
-      <c r="N91" s="15"/>
+      <c r="A91" s="20"/>
+      <c r="B91" s="21"/>
+      <c r="C91" s="21"/>
+      <c r="D91" s="21"/>
+      <c r="E91" s="21"/>
+      <c r="F91" s="22"/>
+      <c r="G91" s="21"/>
+      <c r="H91" s="21"/>
+      <c r="I91" s="21"/>
+      <c r="J91" s="21"/>
+      <c r="K91" s="21"/>
+      <c r="L91" s="21"/>
+      <c r="M91" s="21"/>
+      <c r="N91" s="21"/>
     </row>
     <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="19.5">
-      <c r="A92" s="14"/>
-      <c r="B92" s="15"/>
-      <c r="C92" s="15"/>
-      <c r="D92" s="15"/>
-      <c r="E92" s="15"/>
-      <c r="F92" s="16"/>
-      <c r="G92" s="15"/>
-      <c r="H92" s="15"/>
-      <c r="I92" s="15"/>
-      <c r="J92" s="15"/>
-      <c r="K92" s="15"/>
-      <c r="L92" s="15"/>
-      <c r="M92" s="15"/>
-      <c r="N92" s="15"/>
+      <c r="A92" s="20"/>
+      <c r="B92" s="21"/>
+      <c r="C92" s="21"/>
+      <c r="D92" s="21"/>
+      <c r="E92" s="21"/>
+      <c r="F92" s="22"/>
+      <c r="G92" s="21"/>
+      <c r="H92" s="21"/>
+      <c r="I92" s="21"/>
+      <c r="J92" s="21"/>
+      <c r="K92" s="21"/>
+      <c r="L92" s="21"/>
+      <c r="M92" s="21"/>
+      <c r="N92" s="21"/>
     </row>
     <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="19.5">
-      <c r="A93" s="14"/>
-      <c r="B93" s="15"/>
-      <c r="C93" s="15"/>
-      <c r="D93" s="15"/>
-      <c r="E93" s="15"/>
-      <c r="F93" s="16"/>
-      <c r="G93" s="15"/>
-      <c r="H93" s="15"/>
-      <c r="I93" s="15"/>
-      <c r="J93" s="15"/>
-      <c r="K93" s="15"/>
-      <c r="L93" s="15"/>
-      <c r="M93" s="15"/>
-      <c r="N93" s="15"/>
+      <c r="A93" s="20"/>
+      <c r="B93" s="21"/>
+      <c r="C93" s="21"/>
+      <c r="D93" s="21"/>
+      <c r="E93" s="21"/>
+      <c r="F93" s="22"/>
+      <c r="G93" s="21"/>
+      <c r="H93" s="21"/>
+      <c r="I93" s="21"/>
+      <c r="J93" s="21"/>
+      <c r="K93" s="21"/>
+      <c r="L93" s="21"/>
+      <c r="M93" s="21"/>
+      <c r="N93" s="21"/>
     </row>
     <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="19.5">
-      <c r="A94" s="14"/>
-      <c r="B94" s="15"/>
-      <c r="C94" s="15"/>
-      <c r="D94" s="15"/>
-      <c r="E94" s="15"/>
-      <c r="F94" s="16"/>
-      <c r="G94" s="15"/>
-      <c r="H94" s="15"/>
-      <c r="I94" s="15"/>
-      <c r="J94" s="15"/>
-      <c r="K94" s="15"/>
-      <c r="L94" s="15"/>
-      <c r="M94" s="15"/>
-      <c r="N94" s="15"/>
+      <c r="A94" s="20"/>
+      <c r="B94" s="21"/>
+      <c r="C94" s="21"/>
+      <c r="D94" s="21"/>
+      <c r="E94" s="21"/>
+      <c r="F94" s="22"/>
+      <c r="G94" s="21"/>
+      <c r="H94" s="21"/>
+      <c r="I94" s="21"/>
+      <c r="J94" s="21"/>
+      <c r="K94" s="21"/>
+      <c r="L94" s="21"/>
+      <c r="M94" s="21"/>
+      <c r="N94" s="21"/>
     </row>
     <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="19.5">
-      <c r="A95" s="14"/>
-      <c r="B95" s="15"/>
-      <c r="C95" s="15"/>
-      <c r="D95" s="15"/>
-      <c r="E95" s="15"/>
-      <c r="F95" s="16"/>
-      <c r="G95" s="15"/>
-      <c r="H95" s="15"/>
-      <c r="I95" s="15"/>
-      <c r="J95" s="15"/>
-      <c r="K95" s="15"/>
-      <c r="L95" s="15"/>
-      <c r="M95" s="15"/>
-      <c r="N95" s="15"/>
+      <c r="A95" s="20"/>
+      <c r="B95" s="21"/>
+      <c r="C95" s="21"/>
+      <c r="D95" s="21"/>
+      <c r="E95" s="21"/>
+      <c r="F95" s="22"/>
+      <c r="G95" s="21"/>
+      <c r="H95" s="21"/>
+      <c r="I95" s="21"/>
+      <c r="J95" s="21"/>
+      <c r="K95" s="21"/>
+      <c r="L95" s="21"/>
+      <c r="M95" s="21"/>
+      <c r="N95" s="21"/>
     </row>
     <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="19.5">
-      <c r="A96" s="14"/>
-      <c r="B96" s="15"/>
-      <c r="C96" s="15"/>
-      <c r="D96" s="15"/>
-      <c r="E96" s="15"/>
-      <c r="F96" s="16"/>
-      <c r="G96" s="15"/>
-      <c r="H96" s="15"/>
-      <c r="I96" s="15"/>
-      <c r="J96" s="15"/>
-      <c r="K96" s="15"/>
-      <c r="L96" s="15"/>
-      <c r="M96" s="15"/>
-      <c r="N96" s="15"/>
+      <c r="A96" s="20"/>
+      <c r="B96" s="21"/>
+      <c r="C96" s="21"/>
+      <c r="D96" s="21"/>
+      <c r="E96" s="21"/>
+      <c r="F96" s="22"/>
+      <c r="G96" s="21"/>
+      <c r="H96" s="21"/>
+      <c r="I96" s="21"/>
+      <c r="J96" s="21"/>
+      <c r="K96" s="21"/>
+      <c r="L96" s="21"/>
+      <c r="M96" s="21"/>
+      <c r="N96" s="21"/>
     </row>
     <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="19.5">
-      <c r="A97" s="14"/>
-      <c r="B97" s="15"/>
-      <c r="C97" s="15"/>
-      <c r="D97" s="15"/>
-      <c r="E97" s="15"/>
-      <c r="F97" s="16"/>
-      <c r="G97" s="15"/>
-      <c r="H97" s="15"/>
-      <c r="I97" s="15"/>
-      <c r="J97" s="15"/>
-      <c r="K97" s="15"/>
-      <c r="L97" s="15"/>
-      <c r="M97" s="15"/>
-      <c r="N97" s="15"/>
+      <c r="A97" s="20"/>
+      <c r="B97" s="21"/>
+      <c r="C97" s="21"/>
+      <c r="D97" s="21"/>
+      <c r="E97" s="21"/>
+      <c r="F97" s="22"/>
+      <c r="G97" s="21"/>
+      <c r="H97" s="21"/>
+      <c r="I97" s="21"/>
+      <c r="J97" s="21"/>
+      <c r="K97" s="21"/>
+      <c r="L97" s="21"/>
+      <c r="M97" s="21"/>
+      <c r="N97" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>